<commit_message>
Subir prueba ROI 80%
</commit_message>
<xml_diff>
--- a/resultados/experimentos_entrenamiento.xlsx
+++ b/resultados/experimentos_entrenamiento.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CW6"/>
+  <dimension ref="A1:CW7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2634,11 +2634,358 @@
       <c r="CU6" t="n">
         <v>1</v>
       </c>
-      <c r="CV6" t="b">
+      <c r="CV6" t="n">
         <v>1</v>
       </c>
       <c r="CW6" t="n">
         <v>0.6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:53:46</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>49.10522223313649</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>/Users/luisazcoitipena/Desktop/Repo TFM/TFM-UNIR/models/resnet50_v4_best.pth</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>/Users/luisazcoitipena/Desktop/Repo TFM/TFM-UNIR/resultados/experimentos_entrenamiento.xlsx</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>20</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0.7819181429444105</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>{"Control": 0, "PD": 1}</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>300</v>
+      </c>
+      <c r="N7" t="n">
+        <v>65</v>
+      </c>
+      <c r="O7" t="n">
+        <v>65</v>
+      </c>
+      <c r="P7" t="n">
+        <v>14968834</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>23512130</v>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>data_index.csv</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>data/PPMI_Procesado_2D_Atlas</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>models</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>resultados/experimentos_entrenamiento.xlsx</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>['Control', 'PD']</t>
+        </is>
+      </c>
+      <c r="W7" t="n">
+        <v>2</v>
+      </c>
+      <c r="X7" t="n">
+        <v>60</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>32</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1e-07</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>adamw</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>plateau</t>
+        </is>
+      </c>
+      <c r="AE7" t="n">
+        <v>3</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="AH7" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>layer4</t>
+        </is>
+      </c>
+      <c r="AK7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="b">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>42</v>
+      </c>
+      <c r="AN7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="AQ7" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="AR7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0.1046691254873449</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0.9600417318727178</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>0.9602961349148713</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0.9873006914068012</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0.9598079561042524</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0.9733602281421715</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0.894942225310844</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.8935157085181951</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>9585</v>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>[[2205, 90], [293, 6997]]</t>
+        </is>
+      </c>
+      <c r="BC7" t="n">
+        <v>0.9931630460445116</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>0.9978255784916257</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0.9607843137254902</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0.9598079561042524</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>2205</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>90</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>293</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>6997</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>2.848084348367658</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>0.6525547445255474</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>0.469890873015873</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>0.7533843437316068</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>0.8126984126984127</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>0.7819181429444105</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>-0.06732360578353389</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>-0.06615948031564711</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>2055</v>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>[[61, 419], [295, 1280]]</t>
+        </is>
+      </c>
+      <c r="BU7" t="n">
+        <v>0.4365085978835979</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>0.7368814774309924</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>0.1270833333333333</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>0.8126984126984127</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>61</v>
+      </c>
+      <c r="BZ7" t="n">
+        <v>419</v>
+      </c>
+      <c r="CA7" t="n">
+        <v>295</v>
+      </c>
+      <c r="CB7" t="n">
+        <v>1280</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>2.210545391003871</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>0.6982968369829684</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>0.5392385392385393</v>
+      </c>
+      <c r="CF7" t="n">
+        <v>0.7764705882352941</v>
+      </c>
+      <c r="CG7" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="CH7" t="n">
+        <v>0.8098159509202454</v>
+      </c>
+      <c r="CI7" t="n">
+        <v>0.08877058630943896</v>
+      </c>
+      <c r="CJ7" t="n">
+        <v>0.08686304020640723</v>
+      </c>
+      <c r="CK7" t="n">
+        <v>2055</v>
+      </c>
+      <c r="CL7" t="inlineStr">
+        <is>
+          <t>[[115, 380], [240, 1320]]</t>
+        </is>
+      </c>
+      <c r="CM7" t="n">
+        <v>0.5719289044289044</v>
+      </c>
+      <c r="CN7" t="n">
+        <v>0.8000350332739663</v>
+      </c>
+      <c r="CO7" t="n">
+        <v>0.2323232323232323</v>
+      </c>
+      <c r="CP7" t="n">
+        <v>0.8461538461538461</v>
+      </c>
+      <c r="CQ7" t="n">
+        <v>115</v>
+      </c>
+      <c r="CR7" t="n">
+        <v>380</v>
+      </c>
+      <c r="CS7" t="n">
+        <v>240</v>
+      </c>
+      <c r="CT7" t="n">
+        <v>1320</v>
+      </c>
+      <c r="CU7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CV7" t="n">
+        <v>1</v>
+      </c>
+      <c r="CW7" t="n">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -2652,7 +2999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ75"/>
+  <dimension ref="A1:AQ103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13304,6 +13651,3954 @@
       </c>
       <c r="AQ75" t="n">
         <v>1238</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>0.6483050847457628</v>
+      </c>
+      <c r="G76" t="b">
+        <v>1</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0.6669835724181412</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0.6042775169535733</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0.5910191236988622</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.8184301584410855</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.6164609053497943</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0.7032313590485878</v>
+      </c>
+      <c r="N76" t="n">
+        <v>0.1570428302892106</v>
+      </c>
+      <c r="O76" t="n">
+        <v>0.1435009525384594</v>
+      </c>
+      <c r="P76" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q76" t="inlineStr">
+        <is>
+          <t>[[1298, 997], [2796, 4494]]</t>
+        </is>
+      </c>
+      <c r="R76" t="n">
+        <v>0.6276233895478631</v>
+      </c>
+      <c r="S76" t="n">
+        <v>0.8357151174824824</v>
+      </c>
+      <c r="T76" t="n">
+        <v>0.5655773420479303</v>
+      </c>
+      <c r="U76" t="n">
+        <v>0.6164609053497943</v>
+      </c>
+      <c r="V76" t="n">
+        <v>1298</v>
+      </c>
+      <c r="W76" t="n">
+        <v>997</v>
+      </c>
+      <c r="X76" t="n">
+        <v>2796</v>
+      </c>
+      <c r="Y76" t="n">
+        <v>4494</v>
+      </c>
+      <c r="Z76" t="n">
+        <v>0.7813837033118645</v>
+      </c>
+      <c r="AA76" t="n">
+        <v>0.5153284671532846</v>
+      </c>
+      <c r="AB76" t="n">
+        <v>0.4383035714285715</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>0.7303102625298329</v>
+      </c>
+      <c r="AD76" t="n">
+        <v>0.5828571428571429</v>
+      </c>
+      <c r="AE76" t="n">
+        <v>0.6483050847457628</v>
+      </c>
+      <c r="AF76" t="n">
+        <v>-0.1071227797148469</v>
+      </c>
+      <c r="AG76" t="n">
+        <v>-0.1002951279694229</v>
+      </c>
+      <c r="AH76" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI76" t="inlineStr">
+        <is>
+          <t>[[141, 339], [657, 918]]</t>
+        </is>
+      </c>
+      <c r="AJ76" t="n">
+        <v>0.4226521164021164</v>
+      </c>
+      <c r="AK76" t="n">
+        <v>0.7227060530730315</v>
+      </c>
+      <c r="AL76" t="n">
+        <v>0.29375</v>
+      </c>
+      <c r="AM76" t="n">
+        <v>0.5828571428571429</v>
+      </c>
+      <c r="AN76" t="n">
+        <v>141</v>
+      </c>
+      <c r="AO76" t="n">
+        <v>339</v>
+      </c>
+      <c r="AP76" t="n">
+        <v>657</v>
+      </c>
+      <c r="AQ76" t="n">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>0.6232902033271719</v>
+      </c>
+      <c r="G77" t="b">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0.5823610306345801</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0.6864893062076161</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0.6873113854595336</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0.8750218799229826</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0.6857338820301784</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0.768899484734292</v>
+      </c>
+      <c r="N77" t="n">
+        <v>0.3257988106606056</v>
+      </c>
+      <c r="O77" t="n">
+        <v>0.3032373313651787</v>
+      </c>
+      <c r="P77" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q77" t="inlineStr">
+        <is>
+          <t>[[1581, 714], [2291, 4999]]</t>
+        </is>
+      </c>
+      <c r="R77" t="n">
+        <v>0.7596029419236068</v>
+      </c>
+      <c r="S77" t="n">
+        <v>0.9049432629503308</v>
+      </c>
+      <c r="T77" t="n">
+        <v>0.6888888888888889</v>
+      </c>
+      <c r="U77" t="n">
+        <v>0.6857338820301784</v>
+      </c>
+      <c r="V77" t="n">
+        <v>1581</v>
+      </c>
+      <c r="W77" t="n">
+        <v>714</v>
+      </c>
+      <c r="X77" t="n">
+        <v>2291</v>
+      </c>
+      <c r="Y77" t="n">
+        <v>4999</v>
+      </c>
+      <c r="Z77" t="n">
+        <v>0.8905277867676857</v>
+      </c>
+      <c r="AA77" t="n">
+        <v>0.5041362530413626</v>
+      </c>
+      <c r="AB77" t="n">
+        <v>0.4686607142857143</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>0.7460176991150442</v>
+      </c>
+      <c r="AD77" t="n">
+        <v>0.5352380952380953</v>
+      </c>
+      <c r="AE77" t="n">
+        <v>0.6232902033271719</v>
+      </c>
+      <c r="AF77" t="n">
+        <v>-0.05330523951556161</v>
+      </c>
+      <c r="AG77" t="n">
+        <v>-0.04740218329144308</v>
+      </c>
+      <c r="AH77" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI77" t="inlineStr">
+        <is>
+          <t>[[193, 287], [732, 843]]</t>
+        </is>
+      </c>
+      <c r="AJ77" t="n">
+        <v>0.4435066137566138</v>
+      </c>
+      <c r="AK77" t="n">
+        <v>0.7298523459478771</v>
+      </c>
+      <c r="AL77" t="n">
+        <v>0.4020833333333333</v>
+      </c>
+      <c r="AM77" t="n">
+        <v>0.5352380952380953</v>
+      </c>
+      <c r="AN77" t="n">
+        <v>193</v>
+      </c>
+      <c r="AO77" t="n">
+        <v>287</v>
+      </c>
+      <c r="AP77" t="n">
+        <v>732</v>
+      </c>
+      <c r="AQ77" t="n">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>3</v>
+      </c>
+      <c r="D78" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>0.6925151719487526</v>
+      </c>
+      <c r="G78" t="b">
+        <v>1</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0.4941899075754372</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0.7486697965571205</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0.7569999193092876</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.9120378186729697</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0.7410150891632373</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0.8176795580110497</v>
+      </c>
+      <c r="N78" t="n">
+        <v>0.4514275453103806</v>
+      </c>
+      <c r="O78" t="n">
+        <v>0.4268879067414112</v>
+      </c>
+      <c r="P78" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>[[1774, 521], [1888, 5402]]</t>
+        </is>
+      </c>
+      <c r="R78" t="n">
+        <v>0.8383802983165527</v>
+      </c>
+      <c r="S78" t="n">
+        <v>0.9410435841668356</v>
+      </c>
+      <c r="T78" t="n">
+        <v>0.7729847494553377</v>
+      </c>
+      <c r="U78" t="n">
+        <v>0.7410150891632373</v>
+      </c>
+      <c r="V78" t="n">
+        <v>1774</v>
+      </c>
+      <c r="W78" t="n">
+        <v>521</v>
+      </c>
+      <c r="X78" t="n">
+        <v>1888</v>
+      </c>
+      <c r="Y78" t="n">
+        <v>5402</v>
+      </c>
+      <c r="Z78" t="n">
+        <v>1.161944944841148</v>
+      </c>
+      <c r="AA78" t="n">
+        <v>0.5562043795620438</v>
+      </c>
+      <c r="AB78" t="n">
+        <v>0.4468650793650794</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>0.7383177570093458</v>
+      </c>
+      <c r="AD78" t="n">
+        <v>0.652063492063492</v>
+      </c>
+      <c r="AE78" t="n">
+        <v>0.6925151719487526</v>
+      </c>
+      <c r="AF78" t="n">
+        <v>-0.09614425199597178</v>
+      </c>
+      <c r="AG78" t="n">
+        <v>-0.09377407381469283</v>
+      </c>
+      <c r="AH78" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI78" t="inlineStr">
+        <is>
+          <t>[[116, 364], [548, 1027]]</t>
+        </is>
+      </c>
+      <c r="AJ78" t="n">
+        <v>0.4129193121693122</v>
+      </c>
+      <c r="AK78" t="n">
+        <v>0.7207167099612214</v>
+      </c>
+      <c r="AL78" t="n">
+        <v>0.2416666666666667</v>
+      </c>
+      <c r="AM78" t="n">
+        <v>0.652063492063492</v>
+      </c>
+      <c r="AN78" t="n">
+        <v>116</v>
+      </c>
+      <c r="AO78" t="n">
+        <v>364</v>
+      </c>
+      <c r="AP78" t="n">
+        <v>548</v>
+      </c>
+      <c r="AQ78" t="n">
+        <v>1027</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>4</v>
+      </c>
+      <c r="D79" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>0.6668979875086746</v>
+      </c>
+      <c r="G79" t="b">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0.4250749164312907</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0.7962441314553991</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0.7990236423787622</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.9279871692060946</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.7936899862825789</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0.8556007393715342</v>
+      </c>
+      <c r="N79" t="n">
+        <v>0.5352417717387431</v>
+      </c>
+      <c r="O79" t="n">
+        <v>0.5166768329876785</v>
+      </c>
+      <c r="P79" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>[[1846, 449], [1504, 5786]]</t>
+        </is>
+      </c>
+      <c r="R79" t="n">
+        <v>0.8856238139212399</v>
+      </c>
+      <c r="S79" t="n">
+        <v>0.9580827502489999</v>
+      </c>
+      <c r="T79" t="n">
+        <v>0.8043572984749455</v>
+      </c>
+      <c r="U79" t="n">
+        <v>0.7936899862825789</v>
+      </c>
+      <c r="V79" t="n">
+        <v>1846</v>
+      </c>
+      <c r="W79" t="n">
+        <v>449</v>
+      </c>
+      <c r="X79" t="n">
+        <v>1504</v>
+      </c>
+      <c r="Y79" t="n">
+        <v>5786</v>
+      </c>
+      <c r="Z79" t="n">
+        <v>1.27950052252071</v>
+      </c>
+      <c r="AA79" t="n">
+        <v>0.5328467153284672</v>
+      </c>
+      <c r="AB79" t="n">
+        <v>0.4446626984126984</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>0.7352716143840857</v>
+      </c>
+      <c r="AD79" t="n">
+        <v>0.6101587301587301</v>
+      </c>
+      <c r="AE79" t="n">
+        <v>0.6668979875086746</v>
+      </c>
+      <c r="AF79" t="n">
+        <v>-0.09732407360618489</v>
+      </c>
+      <c r="AG79" t="n">
+        <v>-0.0926855205875512</v>
+      </c>
+      <c r="AH79" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI79" t="inlineStr">
+        <is>
+          <t>[[134, 346], [614, 961]]</t>
+        </is>
+      </c>
+      <c r="AJ79" t="n">
+        <v>0.4368214285714286</v>
+      </c>
+      <c r="AK79" t="n">
+        <v>0.7360402142321639</v>
+      </c>
+      <c r="AL79" t="n">
+        <v>0.2791666666666667</v>
+      </c>
+      <c r="AM79" t="n">
+        <v>0.6101587301587301</v>
+      </c>
+      <c r="AN79" t="n">
+        <v>134</v>
+      </c>
+      <c r="AO79" t="n">
+        <v>346</v>
+      </c>
+      <c r="AP79" t="n">
+        <v>614</v>
+      </c>
+      <c r="AQ79" t="n">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>5</v>
+      </c>
+      <c r="D80" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>0.7137203166226913</v>
+      </c>
+      <c r="G80" t="b">
+        <v>1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0.3711719621235216</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0.8309859154929577</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0.8294763172758816</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.9384472626043922</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0.8323731138545953</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0.8822332073277116</v>
+      </c>
+      <c r="N80" t="n">
+        <v>0.6001831108997882</v>
+      </c>
+      <c r="O80" t="n">
+        <v>0.5867762656818084</v>
+      </c>
+      <c r="P80" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>[[1897, 398], [1222, 6068]]</t>
+        </is>
+      </c>
+      <c r="R80" t="n">
+        <v>0.9144220602430883</v>
+      </c>
+      <c r="S80" t="n">
+        <v>0.9695774628261189</v>
+      </c>
+      <c r="T80" t="n">
+        <v>0.8265795206971678</v>
+      </c>
+      <c r="U80" t="n">
+        <v>0.8323731138545953</v>
+      </c>
+      <c r="V80" t="n">
+        <v>1897</v>
+      </c>
+      <c r="W80" t="n">
+        <v>398</v>
+      </c>
+      <c r="X80" t="n">
+        <v>1222</v>
+      </c>
+      <c r="Y80" t="n">
+        <v>6068</v>
+      </c>
+      <c r="Z80" t="n">
+        <v>1.331898348522882</v>
+      </c>
+      <c r="AA80" t="n">
+        <v>0.5776155717761557</v>
+      </c>
+      <c r="AB80" t="n">
+        <v>0.4528670634920635</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>0.7426218256691832</v>
+      </c>
+      <c r="AD80" t="n">
+        <v>0.686984126984127</v>
+      </c>
+      <c r="AE80" t="n">
+        <v>0.7137203166226913</v>
+      </c>
+      <c r="AF80" t="n">
+        <v>-0.087808189749267</v>
+      </c>
+      <c r="AG80" t="n">
+        <v>-0.08684446231743648</v>
+      </c>
+      <c r="AH80" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI80" t="inlineStr">
+        <is>
+          <t>[[105, 375], [493, 1082]]</t>
+        </is>
+      </c>
+      <c r="AJ80" t="n">
+        <v>0.4378055555555556</v>
+      </c>
+      <c r="AK80" t="n">
+        <v>0.7298162479795007</v>
+      </c>
+      <c r="AL80" t="n">
+        <v>0.21875</v>
+      </c>
+      <c r="AM80" t="n">
+        <v>0.686984126984127</v>
+      </c>
+      <c r="AN80" t="n">
+        <v>105</v>
+      </c>
+      <c r="AO80" t="n">
+        <v>375</v>
+      </c>
+      <c r="AP80" t="n">
+        <v>493</v>
+      </c>
+      <c r="AQ80" t="n">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>0.7095064590924147</v>
+      </c>
+      <c r="G81" t="b">
+        <v>0</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0.3243904571515791</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0.8577986437141367</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0.8574033728717825</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.9500379650721337</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.858161865569273</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0.9017657657657657</v>
+      </c>
+      <c r="N81" t="n">
+        <v>0.6578172145663022</v>
+      </c>
+      <c r="O81" t="n">
+        <v>0.6467429593531548</v>
+      </c>
+      <c r="P81" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>[[1966, 329], [1034, 6256]]</t>
+        </is>
+      </c>
+      <c r="R81" t="n">
+        <v>0.9357648433554187</v>
+      </c>
+      <c r="S81" t="n">
+        <v>0.977487445858443</v>
+      </c>
+      <c r="T81" t="n">
+        <v>0.856644880174292</v>
+      </c>
+      <c r="U81" t="n">
+        <v>0.858161865569273</v>
+      </c>
+      <c r="V81" t="n">
+        <v>1966</v>
+      </c>
+      <c r="W81" t="n">
+        <v>329</v>
+      </c>
+      <c r="X81" t="n">
+        <v>1034</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>6256</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>1.630024549850872</v>
+      </c>
+      <c r="AA81" t="n">
+        <v>0.5732360097323601</v>
+      </c>
+      <c r="AB81" t="n">
+        <v>0.4514583333333334</v>
+      </c>
+      <c r="AC81" t="n">
+        <v>0.7416897506925207</v>
+      </c>
+      <c r="AD81" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AE81" t="n">
+        <v>0.7095064590924147</v>
+      </c>
+      <c r="AF81" t="n">
+        <v>-0.08986723409651358</v>
+      </c>
+      <c r="AG81" t="n">
+        <v>-0.08867102199106602</v>
+      </c>
+      <c r="AH81" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI81" t="inlineStr">
+        <is>
+          <t>[[107, 373], [504, 1071]]</t>
+        </is>
+      </c>
+      <c r="AJ81" t="n">
+        <v>0.4331256613756614</v>
+      </c>
+      <c r="AK81" t="n">
+        <v>0.7313375857525726</v>
+      </c>
+      <c r="AL81" t="n">
+        <v>0.2229166666666667</v>
+      </c>
+      <c r="AM81" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AN81" t="n">
+        <v>107</v>
+      </c>
+      <c r="AO81" t="n">
+        <v>373</v>
+      </c>
+      <c r="AP81" t="n">
+        <v>504</v>
+      </c>
+      <c r="AQ81" t="n">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>7</v>
+      </c>
+      <c r="D82" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>0.7242611237414746</v>
+      </c>
+      <c r="G82" t="b">
+        <v>1</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0.2979517526407695</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0.8672926447574335</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0.8682724118453966</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.9549440580586634</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.8663923182441701</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0.9085155350978136</v>
+      </c>
+      <c r="N82" t="n">
+        <v>0.6796273842915147</v>
+      </c>
+      <c r="O82" t="n">
+        <v>0.6690316338796212</v>
+      </c>
+      <c r="P82" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>[[1997, 298], [974, 6316]]</t>
+        </is>
+      </c>
+      <c r="R82" t="n">
+        <v>0.9456877687822577</v>
+      </c>
+      <c r="S82" t="n">
+        <v>0.9816174202404695</v>
+      </c>
+      <c r="T82" t="n">
+        <v>0.8701525054466231</v>
+      </c>
+      <c r="U82" t="n">
+        <v>0.8663923182441701</v>
+      </c>
+      <c r="V82" t="n">
+        <v>1997</v>
+      </c>
+      <c r="W82" t="n">
+        <v>298</v>
+      </c>
+      <c r="X82" t="n">
+        <v>974</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>6316</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>1.705257742016275</v>
+      </c>
+      <c r="AA82" t="n">
+        <v>0.5868613138686132</v>
+      </c>
+      <c r="AB82" t="n">
+        <v>0.4487599206349207</v>
+      </c>
+      <c r="AC82" t="n">
+        <v>0.7413563829787234</v>
+      </c>
+      <c r="AD82" t="n">
+        <v>0.707936507936508</v>
+      </c>
+      <c r="AE82" t="n">
+        <v>0.7242611237414746</v>
+      </c>
+      <c r="AF82" t="n">
+        <v>-0.09788157966394878</v>
+      </c>
+      <c r="AG82" t="n">
+        <v>-0.09746846192313852</v>
+      </c>
+      <c r="AH82" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI82" t="inlineStr">
+        <is>
+          <t>[[91, 389], [460, 1115]]</t>
+        </is>
+      </c>
+      <c r="AJ82" t="n">
+        <v>0.4177513227513228</v>
+      </c>
+      <c r="AK82" t="n">
+        <v>0.7216880040967752</v>
+      </c>
+      <c r="AL82" t="n">
+        <v>0.1895833333333333</v>
+      </c>
+      <c r="AM82" t="n">
+        <v>0.707936507936508</v>
+      </c>
+      <c r="AN82" t="n">
+        <v>91</v>
+      </c>
+      <c r="AO82" t="n">
+        <v>389</v>
+      </c>
+      <c r="AP82" t="n">
+        <v>460</v>
+      </c>
+      <c r="AQ82" t="n">
+        <v>1115</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>8</v>
+      </c>
+      <c r="D83" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>0.7270358306188925</v>
+      </c>
+      <c r="G83" t="b">
+        <v>1</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0.248639607588077</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0.8906624934793949</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0.8933389816832082</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.9652653548002386</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0.8882030178326474</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0.9251321617373911</v>
+      </c>
+      <c r="N83" t="n">
+        <v>0.7324629064580923</v>
+      </c>
+      <c r="O83" t="n">
+        <v>0.7237948877851771</v>
+      </c>
+      <c r="P83" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q83" t="inlineStr">
+        <is>
+          <t>[[2062, 233], [815, 6475]]</t>
+        </is>
+      </c>
+      <c r="R83" t="n">
+        <v>0.962455687350386</v>
+      </c>
+      <c r="S83" t="n">
+        <v>0.9876040606070442</v>
+      </c>
+      <c r="T83" t="n">
+        <v>0.8984749455337691</v>
+      </c>
+      <c r="U83" t="n">
+        <v>0.8882030178326474</v>
+      </c>
+      <c r="V83" t="n">
+        <v>2062</v>
+      </c>
+      <c r="W83" t="n">
+        <v>233</v>
+      </c>
+      <c r="X83" t="n">
+        <v>815</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>6475</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>1.907690068173002</v>
+      </c>
+      <c r="AA83" t="n">
+        <v>0.5922141119221411</v>
+      </c>
+      <c r="AB83" t="n">
+        <v>0.4594940476190476</v>
+      </c>
+      <c r="AC83" t="n">
+        <v>0.7464882943143812</v>
+      </c>
+      <c r="AD83" t="n">
+        <v>0.7085714285714285</v>
+      </c>
+      <c r="AE83" t="n">
+        <v>0.7270358306188925</v>
+      </c>
+      <c r="AF83" t="n">
+        <v>-0.07698305317899042</v>
+      </c>
+      <c r="AG83" t="n">
+        <v>-0.07657539384846213</v>
+      </c>
+      <c r="AH83" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI83" t="inlineStr">
+        <is>
+          <t>[[101, 379], [459, 1116]]</t>
+        </is>
+      </c>
+      <c r="AJ83" t="n">
+        <v>0.4364854497354498</v>
+      </c>
+      <c r="AK83" t="n">
+        <v>0.7397791397135249</v>
+      </c>
+      <c r="AL83" t="n">
+        <v>0.2104166666666667</v>
+      </c>
+      <c r="AM83" t="n">
+        <v>0.7085714285714285</v>
+      </c>
+      <c r="AN83" t="n">
+        <v>101</v>
+      </c>
+      <c r="AO83" t="n">
+        <v>379</v>
+      </c>
+      <c r="AP83" t="n">
+        <v>459</v>
+      </c>
+      <c r="AQ83" t="n">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>9</v>
+      </c>
+      <c r="D84" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>0.6920762286860582</v>
+      </c>
+      <c r="G84" t="b">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0.2318415988763298</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0.9003651538862807</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0.9006132494149923</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.9665635586978937</v>
+      </c>
+      <c r="L84" t="n">
+        <v>0.9001371742112483</v>
+      </c>
+      <c r="M84" t="n">
+        <v>0.932168477874849</v>
+      </c>
+      <c r="N84" t="n">
+        <v>0.7522096929538417</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0.7454738604413713</v>
+      </c>
+      <c r="P84" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q84" t="inlineStr">
+        <is>
+          <t>[[2068, 227], [728, 6562]]</t>
+        </is>
+      </c>
+      <c r="R84" t="n">
+        <v>0.9675011879466007</v>
+      </c>
+      <c r="S84" t="n">
+        <v>0.9891781052102058</v>
+      </c>
+      <c r="T84" t="n">
+        <v>0.9010893246187364</v>
+      </c>
+      <c r="U84" t="n">
+        <v>0.9001371742112483</v>
+      </c>
+      <c r="V84" t="n">
+        <v>2068</v>
+      </c>
+      <c r="W84" t="n">
+        <v>227</v>
+      </c>
+      <c r="X84" t="n">
+        <v>728</v>
+      </c>
+      <c r="Y84" t="n">
+        <v>6562</v>
+      </c>
+      <c r="Z84" t="n">
+        <v>1.945350923329374</v>
+      </c>
+      <c r="AA84" t="n">
+        <v>0.5518248175182482</v>
+      </c>
+      <c r="AB84" t="n">
+        <v>0.4316964285714285</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>0.7309322033898306</v>
+      </c>
+      <c r="AD84" t="n">
+        <v>0.6571428571428571</v>
+      </c>
+      <c r="AE84" t="n">
+        <v>0.6920762286860582</v>
+      </c>
+      <c r="AF84" t="n">
+        <v>-0.1248683146689059</v>
+      </c>
+      <c r="AG84" t="n">
+        <v>-0.122501267714644</v>
+      </c>
+      <c r="AH84" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI84" t="inlineStr">
+        <is>
+          <t>[[99, 381], [540, 1035]]</t>
+        </is>
+      </c>
+      <c r="AJ84" t="n">
+        <v>0.4190939153439154</v>
+      </c>
+      <c r="AK84" t="n">
+        <v>0.7291439721176262</v>
+      </c>
+      <c r="AL84" t="n">
+        <v>0.20625</v>
+      </c>
+      <c r="AM84" t="n">
+        <v>0.6571428571428571</v>
+      </c>
+      <c r="AN84" t="n">
+        <v>99</v>
+      </c>
+      <c r="AO84" t="n">
+        <v>381</v>
+      </c>
+      <c r="AP84" t="n">
+        <v>540</v>
+      </c>
+      <c r="AQ84" t="n">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>10</v>
+      </c>
+      <c r="D85" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>0.6818956699624957</v>
+      </c>
+      <c r="G85" t="b">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0.2131460117085812</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0.9136150234741784</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0.9142499798273219</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.9716788321167883</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0.9130315500685872</v>
+      </c>
+      <c r="M85" t="n">
+        <v>0.9414427157001415</v>
+      </c>
+      <c r="N85" t="n">
+        <v>0.7829312891833154</v>
+      </c>
+      <c r="O85" t="n">
+        <v>0.7774362080714773</v>
+      </c>
+      <c r="P85" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q85" t="inlineStr">
+        <is>
+          <t>[[2101, 194], [634, 6656]]</t>
+        </is>
+      </c>
+      <c r="R85" t="n">
+        <v>0.9723327087274477</v>
+      </c>
+      <c r="S85" t="n">
+        <v>0.9909346682044144</v>
+      </c>
+      <c r="T85" t="n">
+        <v>0.9154684095860567</v>
+      </c>
+      <c r="U85" t="n">
+        <v>0.9130315500685872</v>
+      </c>
+      <c r="V85" t="n">
+        <v>2101</v>
+      </c>
+      <c r="W85" t="n">
+        <v>194</v>
+      </c>
+      <c r="X85" t="n">
+        <v>634</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>6656</v>
+      </c>
+      <c r="Z85" t="n">
+        <v>1.813816284727296</v>
+      </c>
+      <c r="AA85" t="n">
+        <v>0.545985401459854</v>
+      </c>
+      <c r="AB85" t="n">
+        <v>0.4445436507936508</v>
+      </c>
+      <c r="AC85" t="n">
+        <v>0.7363770250368189</v>
+      </c>
+      <c r="AD85" t="n">
+        <v>0.6349206349206349</v>
+      </c>
+      <c r="AE85" t="n">
+        <v>0.6818956699624957</v>
+      </c>
+      <c r="AF85" t="n">
+        <v>-0.09912333265797843</v>
+      </c>
+      <c r="AG85" t="n">
+        <v>-0.0958496583534092</v>
+      </c>
+      <c r="AH85" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI85" t="inlineStr">
+        <is>
+          <t>[[122, 358], [575, 1000]]</t>
+        </is>
+      </c>
+      <c r="AJ85" t="n">
+        <v>0.4297387566137566</v>
+      </c>
+      <c r="AK85" t="n">
+        <v>0.7288434867289292</v>
+      </c>
+      <c r="AL85" t="n">
+        <v>0.2541666666666667</v>
+      </c>
+      <c r="AM85" t="n">
+        <v>0.6349206349206349</v>
+      </c>
+      <c r="AN85" t="n">
+        <v>122</v>
+      </c>
+      <c r="AO85" t="n">
+        <v>358</v>
+      </c>
+      <c r="AP85" t="n">
+        <v>575</v>
+      </c>
+      <c r="AQ85" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>11</v>
+      </c>
+      <c r="D86" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>0.7355584082156611</v>
+      </c>
+      <c r="G86" t="b">
+        <v>1</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0.1950511277106726</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0.9183098591549296</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0.9185306221253933</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.9729611862189271</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0.9181069958847736</v>
+      </c>
+      <c r="M86" t="n">
+        <v>0.9447385136565742</v>
+      </c>
+      <c r="N86" t="n">
+        <v>0.7935710076313962</v>
+      </c>
+      <c r="O86" t="n">
+        <v>0.7886736078641563</v>
+      </c>
+      <c r="P86" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q86" t="inlineStr">
+        <is>
+          <t>[[2109, 186], [597, 6693]]</t>
+        </is>
+      </c>
+      <c r="R86" t="n">
+        <v>0.9770406232909259</v>
+      </c>
+      <c r="S86" t="n">
+        <v>0.9925137033667174</v>
+      </c>
+      <c r="T86" t="n">
+        <v>0.918954248366013</v>
+      </c>
+      <c r="U86" t="n">
+        <v>0.9181069958847736</v>
+      </c>
+      <c r="V86" t="n">
+        <v>2109</v>
+      </c>
+      <c r="W86" t="n">
+        <v>186</v>
+      </c>
+      <c r="X86" t="n">
+        <v>597</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>6693</v>
+      </c>
+      <c r="Z86" t="n">
+        <v>2.178549090151079</v>
+      </c>
+      <c r="AA86" t="n">
+        <v>0.5990267639902677</v>
+      </c>
+      <c r="AB86" t="n">
+        <v>0.4523511904761905</v>
+      </c>
+      <c r="AC86" t="n">
+        <v>0.7436729396495781</v>
+      </c>
+      <c r="AD86" t="n">
+        <v>0.7276190476190476</v>
+      </c>
+      <c r="AE86" t="n">
+        <v>0.7355584082156611</v>
+      </c>
+      <c r="AF86" t="n">
+        <v>-0.09310222693186695</v>
+      </c>
+      <c r="AG86" t="n">
+        <v>-0.09300749404542907</v>
+      </c>
+      <c r="AH86" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI86" t="inlineStr">
+        <is>
+          <t>[[85, 395], [429, 1146]]</t>
+        </is>
+      </c>
+      <c r="AJ86" t="n">
+        <v>0.4182863756613757</v>
+      </c>
+      <c r="AK86" t="n">
+        <v>0.7288493015690738</v>
+      </c>
+      <c r="AL86" t="n">
+        <v>0.1770833333333333</v>
+      </c>
+      <c r="AM86" t="n">
+        <v>0.7276190476190476</v>
+      </c>
+      <c r="AN86" t="n">
+        <v>85</v>
+      </c>
+      <c r="AO86" t="n">
+        <v>395</v>
+      </c>
+      <c r="AP86" t="n">
+        <v>429</v>
+      </c>
+      <c r="AQ86" t="n">
+        <v>1146</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>12</v>
+      </c>
+      <c r="D87" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>0.7029009669889963</v>
+      </c>
+      <c r="G87" t="b">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0.1762225886240376</v>
+      </c>
+      <c r="I87" t="n">
+        <v>0.9300991131977048</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0.9295650770596304</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.9763960852043754</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0.9305898491083676</v>
+      </c>
+      <c r="M87" t="n">
+        <v>0.9529428290490237</v>
+      </c>
+      <c r="N87" t="n">
+        <v>0.8209734296916359</v>
+      </c>
+      <c r="O87" t="n">
+        <v>0.8173994487820233</v>
+      </c>
+      <c r="P87" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q87" t="inlineStr">
+        <is>
+          <t>[[2131, 164], [506, 6784]]</t>
+        </is>
+      </c>
+      <c r="R87" t="n">
+        <v>0.9809498791133585</v>
+      </c>
+      <c r="S87" t="n">
+        <v>0.9937937227967556</v>
+      </c>
+      <c r="T87" t="n">
+        <v>0.9285403050108932</v>
+      </c>
+      <c r="U87" t="n">
+        <v>0.9305898491083676</v>
+      </c>
+      <c r="V87" t="n">
+        <v>2131</v>
+      </c>
+      <c r="W87" t="n">
+        <v>164</v>
+      </c>
+      <c r="X87" t="n">
+        <v>506</v>
+      </c>
+      <c r="Y87" t="n">
+        <v>6784</v>
+      </c>
+      <c r="Z87" t="n">
+        <v>2.010111190860869</v>
+      </c>
+      <c r="AA87" t="n">
+        <v>0.5664233576642336</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>0.4491865079365079</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>0.7401685393258427</v>
+      </c>
+      <c r="AD87" t="n">
+        <v>0.6692063492063492</v>
+      </c>
+      <c r="AE87" t="n">
+        <v>0.7029009669889963</v>
+      </c>
+      <c r="AF87" t="n">
+        <v>-0.09321810309128302</v>
+      </c>
+      <c r="AG87" t="n">
+        <v>-0.09160906074778885</v>
+      </c>
+      <c r="AH87" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI87" t="inlineStr">
+        <is>
+          <t>[[110, 370], [521, 1054]]</t>
+        </is>
+      </c>
+      <c r="AJ87" t="n">
+        <v>0.42807208994709</v>
+      </c>
+      <c r="AK87" t="n">
+        <v>0.736257451747703</v>
+      </c>
+      <c r="AL87" t="n">
+        <v>0.2291666666666667</v>
+      </c>
+      <c r="AM87" t="n">
+        <v>0.6692063492063492</v>
+      </c>
+      <c r="AN87" t="n">
+        <v>110</v>
+      </c>
+      <c r="AO87" t="n">
+        <v>370</v>
+      </c>
+      <c r="AP87" t="n">
+        <v>521</v>
+      </c>
+      <c r="AQ87" t="n">
+        <v>1054</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>13</v>
+      </c>
+      <c r="D88" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>0.7464477423429112</v>
+      </c>
+      <c r="G88" t="b">
+        <v>1</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0.1573841607782078</v>
+      </c>
+      <c r="I88" t="n">
+        <v>0.9371935315597287</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0.9381102235132737</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.9801838024124067</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0.9363511659807956</v>
+      </c>
+      <c r="M88" t="n">
+        <v>0.9577662410551424</v>
+      </c>
+      <c r="N88" t="n">
+        <v>0.838891126938579</v>
+      </c>
+      <c r="O88" t="n">
+        <v>0.835558359815637</v>
+      </c>
+      <c r="P88" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q88" t="inlineStr">
+        <is>
+          <t>[[2157, 138], [464, 6826]]</t>
+        </is>
+      </c>
+      <c r="R88" t="n">
+        <v>0.9849154988927441</v>
+      </c>
+      <c r="S88" t="n">
+        <v>0.9950091617422605</v>
+      </c>
+      <c r="T88" t="n">
+        <v>0.9398692810457516</v>
+      </c>
+      <c r="U88" t="n">
+        <v>0.9363511659807956</v>
+      </c>
+      <c r="V88" t="n">
+        <v>2157</v>
+      </c>
+      <c r="W88" t="n">
+        <v>138</v>
+      </c>
+      <c r="X88" t="n">
+        <v>464</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>6826</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>2.40014597273221</v>
+      </c>
+      <c r="AA88" t="n">
+        <v>0.6092457420924574</v>
+      </c>
+      <c r="AB88" t="n">
+        <v>0.4481547619047619</v>
+      </c>
+      <c r="AC88" t="n">
+        <v>0.742462311557789</v>
+      </c>
+      <c r="AD88" t="n">
+        <v>0.7504761904761905</v>
+      </c>
+      <c r="AE88" t="n">
+        <v>0.7464477423429112</v>
+      </c>
+      <c r="AF88" t="n">
+        <v>-0.1050117121621974</v>
+      </c>
+      <c r="AG88" t="n">
+        <v>-0.1049829749193947</v>
+      </c>
+      <c r="AH88" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI88" t="inlineStr">
+        <is>
+          <t>[[70, 410], [393, 1182]]</t>
+        </is>
+      </c>
+      <c r="AJ88" t="n">
+        <v>0.4283472222222223</v>
+      </c>
+      <c r="AK88" t="n">
+        <v>0.7399948662836526</v>
+      </c>
+      <c r="AL88" t="n">
+        <v>0.1458333333333333</v>
+      </c>
+      <c r="AM88" t="n">
+        <v>0.7504761904761905</v>
+      </c>
+      <c r="AN88" t="n">
+        <v>70</v>
+      </c>
+      <c r="AO88" t="n">
+        <v>410</v>
+      </c>
+      <c r="AP88" t="n">
+        <v>393</v>
+      </c>
+      <c r="AQ88" t="n">
+        <v>1182</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>14</v>
+      </c>
+      <c r="D89" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>0.7288573273079406</v>
+      </c>
+      <c r="G89" t="b">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0.140160233634303</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0.9426186750130412</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0.9419753086419753</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.9806046776953794</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0.9432098765432099</v>
+      </c>
+      <c r="M89" t="n">
+        <v>0.9615438400223745</v>
+      </c>
+      <c r="N89" t="n">
+        <v>0.8512208753198409</v>
+      </c>
+      <c r="O89" t="n">
+        <v>0.8487290138138883</v>
+      </c>
+      <c r="P89" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>[[2159, 136], [414, 6876]]</t>
+        </is>
+      </c>
+      <c r="R89" t="n">
+        <v>0.9881262719994264</v>
+      </c>
+      <c r="S89" t="n">
+        <v>0.9961700990010174</v>
+      </c>
+      <c r="T89" t="n">
+        <v>0.9407407407407408</v>
+      </c>
+      <c r="U89" t="n">
+        <v>0.9432098765432099</v>
+      </c>
+      <c r="V89" t="n">
+        <v>2159</v>
+      </c>
+      <c r="W89" t="n">
+        <v>136</v>
+      </c>
+      <c r="X89" t="n">
+        <v>414</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>6876</v>
+      </c>
+      <c r="Z89" t="n">
+        <v>2.536379545680508</v>
+      </c>
+      <c r="AA89" t="n">
+        <v>0.5912408759124088</v>
+      </c>
+      <c r="AB89" t="n">
+        <v>0.4479960317460318</v>
+      </c>
+      <c r="AC89" t="n">
+        <v>0.7413000656598818</v>
+      </c>
+      <c r="AD89" t="n">
+        <v>0.7168253968253968</v>
+      </c>
+      <c r="AE89" t="n">
+        <v>0.7288573273079406</v>
+      </c>
+      <c r="AF89" t="n">
+        <v>-0.1004665780294039</v>
+      </c>
+      <c r="AG89" t="n">
+        <v>-0.100233278519255</v>
+      </c>
+      <c r="AH89" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI89" t="inlineStr">
+        <is>
+          <t>[[86, 394], [446, 1129]]</t>
+        </is>
+      </c>
+      <c r="AJ89" t="n">
+        <v>0.4118611111111111</v>
+      </c>
+      <c r="AK89" t="n">
+        <v>0.7308304713635989</v>
+      </c>
+      <c r="AL89" t="n">
+        <v>0.1791666666666667</v>
+      </c>
+      <c r="AM89" t="n">
+        <v>0.7168253968253968</v>
+      </c>
+      <c r="AN89" t="n">
+        <v>86</v>
+      </c>
+      <c r="AO89" t="n">
+        <v>394</v>
+      </c>
+      <c r="AP89" t="n">
+        <v>446</v>
+      </c>
+      <c r="AQ89" t="n">
+        <v>1129</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>15</v>
+      </c>
+      <c r="D90" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>0.6714677640603567</v>
+      </c>
+      <c r="G90" t="b">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0.1495579196626965</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0.9437663015127804</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0.9425804889857177</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0.9804982206405694</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0.9448559670781893</v>
+      </c>
+      <c r="M90" t="n">
+        <v>0.9623471882640586</v>
+      </c>
+      <c r="N90" t="n">
+        <v>0.8537568910757802</v>
+      </c>
+      <c r="O90" t="n">
+        <v>0.8514776939048765</v>
+      </c>
+      <c r="P90" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>[[2158, 137], [402, 6888]]</t>
+        </is>
+      </c>
+      <c r="R90" t="n">
+        <v>0.9859437376535739</v>
+      </c>
+      <c r="S90" t="n">
+        <v>0.9951533120875031</v>
+      </c>
+      <c r="T90" t="n">
+        <v>0.9403050108932461</v>
+      </c>
+      <c r="U90" t="n">
+        <v>0.9448559670781893</v>
+      </c>
+      <c r="V90" t="n">
+        <v>2158</v>
+      </c>
+      <c r="W90" t="n">
+        <v>137</v>
+      </c>
+      <c r="X90" t="n">
+        <v>402</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>6888</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>2.153448349193935</v>
+      </c>
+      <c r="AA90" t="n">
+        <v>0.5338199513381995</v>
+      </c>
+      <c r="AB90" t="n">
+        <v>0.4337103174603175</v>
+      </c>
+      <c r="AC90" t="n">
+        <v>0.7300521998508576</v>
+      </c>
+      <c r="AD90" t="n">
+        <v>0.6215873015873016</v>
+      </c>
+      <c r="AE90" t="n">
+        <v>0.6714677640603567</v>
+      </c>
+      <c r="AF90" t="n">
+        <v>-0.1178076079336517</v>
+      </c>
+      <c r="AG90" t="n">
+        <v>-0.1133676048930288</v>
+      </c>
+      <c r="AH90" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI90" t="inlineStr">
+        <is>
+          <t>[[118, 362], [596, 979]]</t>
+        </is>
+      </c>
+      <c r="AJ90" t="n">
+        <v>0.4189973544973545</v>
+      </c>
+      <c r="AK90" t="n">
+        <v>0.732458651813799</v>
+      </c>
+      <c r="AL90" t="n">
+        <v>0.2458333333333333</v>
+      </c>
+      <c r="AM90" t="n">
+        <v>0.6215873015873016</v>
+      </c>
+      <c r="AN90" t="n">
+        <v>118</v>
+      </c>
+      <c r="AO90" t="n">
+        <v>362</v>
+      </c>
+      <c r="AP90" t="n">
+        <v>596</v>
+      </c>
+      <c r="AQ90" t="n">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>16</v>
+      </c>
+      <c r="D91" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>0.7510204081632653</v>
+      </c>
+      <c r="G91" t="b">
+        <v>1</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0.1296287581239073</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0.9497130933750652</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0.9485798434600177</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.982563084774596</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0.9507544581618655</v>
+      </c>
+      <c r="M91" t="n">
+        <v>0.9663970998326826</v>
+      </c>
+      <c r="N91" t="n">
+        <v>0.8684824755262275</v>
+      </c>
+      <c r="O91" t="n">
+        <v>0.8666287335536571</v>
+      </c>
+      <c r="P91" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>[[2172, 123], [359, 6931]]</t>
+        </is>
+      </c>
+      <c r="R91" t="n">
+        <v>0.9897158491502073</v>
+      </c>
+      <c r="S91" t="n">
+        <v>0.9966693276538431</v>
+      </c>
+      <c r="T91" t="n">
+        <v>0.9464052287581699</v>
+      </c>
+      <c r="U91" t="n">
+        <v>0.9507544581618655</v>
+      </c>
+      <c r="V91" t="n">
+        <v>2172</v>
+      </c>
+      <c r="W91" t="n">
+        <v>123</v>
+      </c>
+      <c r="X91" t="n">
+        <v>359</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>6931</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>2.662155884373797</v>
+      </c>
+      <c r="AA91" t="n">
+        <v>0.6141119221411192</v>
+      </c>
+      <c r="AB91" t="n">
+        <v>0.4484325396825397</v>
+      </c>
+      <c r="AC91" t="n">
+        <v>0.7428571428571429</v>
+      </c>
+      <c r="AD91" t="n">
+        <v>0.7593650793650794</v>
+      </c>
+      <c r="AE91" t="n">
+        <v>0.7510204081632653</v>
+      </c>
+      <c r="AF91" t="n">
+        <v>-0.1059433479175248</v>
+      </c>
+      <c r="AG91" t="n">
+        <v>-0.1058170899282407</v>
+      </c>
+      <c r="AH91" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI91" t="inlineStr">
+        <is>
+          <t>[[66, 414], [379, 1196]]</t>
+        </is>
+      </c>
+      <c r="AJ91" t="n">
+        <v>0.4206626984126984</v>
+      </c>
+      <c r="AK91" t="n">
+        <v>0.7402101530431884</v>
+      </c>
+      <c r="AL91" t="n">
+        <v>0.1375</v>
+      </c>
+      <c r="AM91" t="n">
+        <v>0.7593650793650794</v>
+      </c>
+      <c r="AN91" t="n">
+        <v>66</v>
+      </c>
+      <c r="AO91" t="n">
+        <v>414</v>
+      </c>
+      <c r="AP91" t="n">
+        <v>379</v>
+      </c>
+      <c r="AQ91" t="n">
+        <v>1196</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>17</v>
+      </c>
+      <c r="D92" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>0.7462025316455696</v>
+      </c>
+      <c r="G92" t="b">
+        <v>0</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0.1281132510729643</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0.9501304121022431</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0.9491527475187607</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0.9828466118514319</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0.9510288065843622</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0.9666759620747351</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0.8695916585232569</v>
+      </c>
+      <c r="O92" t="n">
+        <v>0.8677355490428384</v>
+      </c>
+      <c r="P92" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>[[2174, 121], [357, 6933]]</t>
+        </is>
+      </c>
+      <c r="R92" t="n">
+        <v>0.9896518046328423</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0.9965173935889351</v>
+      </c>
+      <c r="T92" t="n">
+        <v>0.947276688453159</v>
+      </c>
+      <c r="U92" t="n">
+        <v>0.9510288065843622</v>
+      </c>
+      <c r="V92" t="n">
+        <v>2174</v>
+      </c>
+      <c r="W92" t="n">
+        <v>121</v>
+      </c>
+      <c r="X92" t="n">
+        <v>357</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>6933</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>2.492752975500993</v>
+      </c>
+      <c r="AA92" t="n">
+        <v>0.6097323600973236</v>
+      </c>
+      <c r="AB92" t="n">
+        <v>0.4513690476190476</v>
+      </c>
+      <c r="AC92" t="n">
+        <v>0.7438485804416404</v>
+      </c>
+      <c r="AD92" t="n">
+        <v>0.7485714285714286</v>
+      </c>
+      <c r="AE92" t="n">
+        <v>0.7462025316455696</v>
+      </c>
+      <c r="AF92" t="n">
+        <v>-0.09798060256644844</v>
+      </c>
+      <c r="AG92" t="n">
+        <v>-0.09797142000599579</v>
+      </c>
+      <c r="AH92" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI92" t="inlineStr">
+        <is>
+          <t>[[74, 406], [396, 1179]]</t>
+        </is>
+      </c>
+      <c r="AJ92" t="n">
+        <v>0.4211818783068784</v>
+      </c>
+      <c r="AK92" t="n">
+        <v>0.7443631872322072</v>
+      </c>
+      <c r="AL92" t="n">
+        <v>0.1541666666666667</v>
+      </c>
+      <c r="AM92" t="n">
+        <v>0.7485714285714286</v>
+      </c>
+      <c r="AN92" t="n">
+        <v>74</v>
+      </c>
+      <c r="AO92" t="n">
+        <v>406</v>
+      </c>
+      <c r="AP92" t="n">
+        <v>396</v>
+      </c>
+      <c r="AQ92" t="n">
+        <v>1179</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>18</v>
+      </c>
+      <c r="D93" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>0.7725030826140568</v>
+      </c>
+      <c r="G93" t="b">
+        <v>1</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0.1048569103859338</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0.9605633802816902</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0.9601912369886226</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0.9868977176669484</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.9609053497942387</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0.9737281067556297</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0.8960197019153145</v>
+      </c>
+      <c r="O93" t="n">
+        <v>0.8947380806702123</v>
+      </c>
+      <c r="P93" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>[[2202, 93], [285, 7005]]</t>
+        </is>
+      </c>
+      <c r="R93" t="n">
+        <v>0.9932311250975012</v>
+      </c>
+      <c r="S93" t="n">
+        <v>0.9977772124425429</v>
+      </c>
+      <c r="T93" t="n">
+        <v>0.9594771241830066</v>
+      </c>
+      <c r="U93" t="n">
+        <v>0.9609053497942387</v>
+      </c>
+      <c r="V93" t="n">
+        <v>2202</v>
+      </c>
+      <c r="W93" t="n">
+        <v>93</v>
+      </c>
+      <c r="X93" t="n">
+        <v>285</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>7005</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>2.983440462980247</v>
+      </c>
+      <c r="AA93" t="n">
+        <v>0.6408759124087591</v>
+      </c>
+      <c r="AB93" t="n">
+        <v>0.4644444444444444</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>0.7507489514679448</v>
+      </c>
+      <c r="AD93" t="n">
+        <v>0.7955555555555556</v>
+      </c>
+      <c r="AE93" t="n">
+        <v>0.7725030826140568</v>
+      </c>
+      <c r="AF93" t="n">
+        <v>-0.07703295212887763</v>
+      </c>
+      <c r="AG93" t="n">
+        <v>-0.07630564840639575</v>
+      </c>
+      <c r="AH93" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI93" t="inlineStr">
+        <is>
+          <t>[[64, 416], [322, 1253]]</t>
+        </is>
+      </c>
+      <c r="AJ93" t="n">
+        <v>0.4138730158730158</v>
+      </c>
+      <c r="AK93" t="n">
+        <v>0.7288776854297443</v>
+      </c>
+      <c r="AL93" t="n">
+        <v>0.1333333333333333</v>
+      </c>
+      <c r="AM93" t="n">
+        <v>0.7955555555555556</v>
+      </c>
+      <c r="AN93" t="n">
+        <v>64</v>
+      </c>
+      <c r="AO93" t="n">
+        <v>416</v>
+      </c>
+      <c r="AP93" t="n">
+        <v>322</v>
+      </c>
+      <c r="AQ93" t="n">
+        <v>1253</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>19</v>
+      </c>
+      <c r="D94" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>0.773838630806846</v>
+      </c>
+      <c r="G94" t="b">
+        <v>1</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0.1149515318233922</v>
+      </c>
+      <c r="I94" t="n">
+        <v>0.9544079290558164</v>
+      </c>
+      <c r="J94" t="n">
+        <v>0.9534575970305817</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0.9843109540636042</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0.955281207133059</v>
+      </c>
+      <c r="M94" t="n">
+        <v>0.9695788374521406</v>
+      </c>
+      <c r="N94" t="n">
+        <v>0.8802817622395146</v>
+      </c>
+      <c r="O94" t="n">
+        <v>0.8787131325371851</v>
+      </c>
+      <c r="P94" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>[[2184, 111], [326, 6964]]</t>
+        </is>
+      </c>
+      <c r="R94" t="n">
+        <v>0.9917518551392511</v>
+      </c>
+      <c r="S94" t="n">
+        <v>0.9972715273942987</v>
+      </c>
+      <c r="T94" t="n">
+        <v>0.9516339869281045</v>
+      </c>
+      <c r="U94" t="n">
+        <v>0.955281207133059</v>
+      </c>
+      <c r="V94" t="n">
+        <v>2184</v>
+      </c>
+      <c r="W94" t="n">
+        <v>111</v>
+      </c>
+      <c r="X94" t="n">
+        <v>326</v>
+      </c>
+      <c r="Y94" t="n">
+        <v>6964</v>
+      </c>
+      <c r="Z94" t="n">
+        <v>2.76323731531482</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>0.6399026763990268</v>
+      </c>
+      <c r="AB94" t="n">
+        <v>0.4529464285714286</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>0.7460223924572775</v>
+      </c>
+      <c r="AD94" t="n">
+        <v>0.8038095238095239</v>
+      </c>
+      <c r="AE94" t="n">
+        <v>0.773838630806846</v>
+      </c>
+      <c r="AF94" t="n">
+        <v>-0.1049786664201807</v>
+      </c>
+      <c r="AG94" t="n">
+        <v>-0.1032276318366814</v>
+      </c>
+      <c r="AH94" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI94" t="inlineStr">
+        <is>
+          <t>[[49, 431], [309, 1266]]</t>
+        </is>
+      </c>
+      <c r="AJ94" t="n">
+        <v>0.4347367724867724</v>
+      </c>
+      <c r="AK94" t="n">
+        <v>0.756686933080595</v>
+      </c>
+      <c r="AL94" t="n">
+        <v>0.1020833333333333</v>
+      </c>
+      <c r="AM94" t="n">
+        <v>0.8038095238095239</v>
+      </c>
+      <c r="AN94" t="n">
+        <v>49</v>
+      </c>
+      <c r="AO94" t="n">
+        <v>431</v>
+      </c>
+      <c r="AP94" t="n">
+        <v>309</v>
+      </c>
+      <c r="AQ94" t="n">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>20</v>
+      </c>
+      <c r="D95" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>0.7819181429444105</v>
+      </c>
+      <c r="G95" t="b">
+        <v>1</v>
+      </c>
+      <c r="H95" t="n">
+        <v>0.1046691254873449</v>
+      </c>
+      <c r="I95" t="n">
+        <v>0.9600417318727178</v>
+      </c>
+      <c r="J95" t="n">
+        <v>0.9602961349148713</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0.9873006914068012</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0.9598079561042524</v>
+      </c>
+      <c r="M95" t="n">
+        <v>0.9733602281421715</v>
+      </c>
+      <c r="N95" t="n">
+        <v>0.894942225310844</v>
+      </c>
+      <c r="O95" t="n">
+        <v>0.8935157085181951</v>
+      </c>
+      <c r="P95" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>[[2205, 90], [293, 6997]]</t>
+        </is>
+      </c>
+      <c r="R95" t="n">
+        <v>0.9931630460445116</v>
+      </c>
+      <c r="S95" t="n">
+        <v>0.9978255784916257</v>
+      </c>
+      <c r="T95" t="n">
+        <v>0.9607843137254902</v>
+      </c>
+      <c r="U95" t="n">
+        <v>0.9598079561042524</v>
+      </c>
+      <c r="V95" t="n">
+        <v>2205</v>
+      </c>
+      <c r="W95" t="n">
+        <v>90</v>
+      </c>
+      <c r="X95" t="n">
+        <v>293</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>6997</v>
+      </c>
+      <c r="Z95" t="n">
+        <v>2.848084348367658</v>
+      </c>
+      <c r="AA95" t="n">
+        <v>0.6525547445255474</v>
+      </c>
+      <c r="AB95" t="n">
+        <v>0.469890873015873</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>0.7533843437316068</v>
+      </c>
+      <c r="AD95" t="n">
+        <v>0.8126984126984127</v>
+      </c>
+      <c r="AE95" t="n">
+        <v>0.7819181429444105</v>
+      </c>
+      <c r="AF95" t="n">
+        <v>-0.06732360578353389</v>
+      </c>
+      <c r="AG95" t="n">
+        <v>-0.06615948031564711</v>
+      </c>
+      <c r="AH95" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI95" t="inlineStr">
+        <is>
+          <t>[[61, 419], [295, 1280]]</t>
+        </is>
+      </c>
+      <c r="AJ95" t="n">
+        <v>0.4365085978835979</v>
+      </c>
+      <c r="AK95" t="n">
+        <v>0.7368814774309924</v>
+      </c>
+      <c r="AL95" t="n">
+        <v>0.1270833333333333</v>
+      </c>
+      <c r="AM95" t="n">
+        <v>0.8126984126984127</v>
+      </c>
+      <c r="AN95" t="n">
+        <v>61</v>
+      </c>
+      <c r="AO95" t="n">
+        <v>419</v>
+      </c>
+      <c r="AP95" t="n">
+        <v>295</v>
+      </c>
+      <c r="AQ95" t="n">
+        <v>1280</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>21</v>
+      </c>
+      <c r="D96" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>0.7268593699253004</v>
+      </c>
+      <c r="G96" t="b">
+        <v>0</v>
+      </c>
+      <c r="H96" t="n">
+        <v>0.08842004945285008</v>
+      </c>
+      <c r="I96" t="n">
+        <v>0.9695357329160146</v>
+      </c>
+      <c r="J96" t="n">
+        <v>0.9692245622528847</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0.9899187902548305</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0.9698216735253772</v>
+      </c>
+      <c r="M96" t="n">
+        <v>0.9797671840354767</v>
+      </c>
+      <c r="N96" t="n">
+        <v>0.9189548753347153</v>
+      </c>
+      <c r="O96" t="n">
+        <v>0.9181640193261124</v>
+      </c>
+      <c r="P96" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q96" t="inlineStr">
+        <is>
+          <t>[[2223, 72], [220, 7070]]</t>
+        </is>
+      </c>
+      <c r="R96" t="n">
+        <v>0.9950056035217013</v>
+      </c>
+      <c r="S96" t="n">
+        <v>0.9983341766635065</v>
+      </c>
+      <c r="T96" t="n">
+        <v>0.9686274509803922</v>
+      </c>
+      <c r="U96" t="n">
+        <v>0.9698216735253772</v>
+      </c>
+      <c r="V96" t="n">
+        <v>2223</v>
+      </c>
+      <c r="W96" t="n">
+        <v>72</v>
+      </c>
+      <c r="X96" t="n">
+        <v>220</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>7070</v>
+      </c>
+      <c r="Z96" t="n">
+        <v>2.830795383917444</v>
+      </c>
+      <c r="AA96" t="n">
+        <v>0.5907542579075425</v>
+      </c>
+      <c r="AB96" t="n">
+        <v>0.4541964285714286</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>0.7440159574468085</v>
+      </c>
+      <c r="AD96" t="n">
+        <v>0.7104761904761905</v>
+      </c>
+      <c r="AE96" t="n">
+        <v>0.7268593699253004</v>
+      </c>
+      <c r="AF96" t="n">
+        <v>-0.0874964672426818</v>
+      </c>
+      <c r="AG96" t="n">
+        <v>-0.08712718077427506</v>
+      </c>
+      <c r="AH96" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI96" t="inlineStr">
+        <is>
+          <t>[[95, 385], [456, 1119]]</t>
+        </is>
+      </c>
+      <c r="AJ96" t="n">
+        <v>0.4279100529100529</v>
+      </c>
+      <c r="AK96" t="n">
+        <v>0.7429521812543172</v>
+      </c>
+      <c r="AL96" t="n">
+        <v>0.1979166666666667</v>
+      </c>
+      <c r="AM96" t="n">
+        <v>0.7104761904761905</v>
+      </c>
+      <c r="AN96" t="n">
+        <v>95</v>
+      </c>
+      <c r="AO96" t="n">
+        <v>385</v>
+      </c>
+      <c r="AP96" t="n">
+        <v>456</v>
+      </c>
+      <c r="AQ96" t="n">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>22</v>
+      </c>
+      <c r="D97" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>0.7510307643514114</v>
+      </c>
+      <c r="G97" t="b">
+        <v>0</v>
+      </c>
+      <c r="H97" t="n">
+        <v>0.0949607235204135</v>
+      </c>
+      <c r="I97" t="n">
+        <v>0.96452790818988</v>
+      </c>
+      <c r="J97" t="n">
+        <v>0.9642903251835714</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0.9883361439010681</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.9647462277091907</v>
+      </c>
+      <c r="M97" t="n">
+        <v>0.9763987227544079</v>
+      </c>
+      <c r="N97" t="n">
+        <v>0.9061419238600115</v>
+      </c>
+      <c r="O97" t="n">
+        <v>0.9050720021392225</v>
+      </c>
+      <c r="P97" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q97" t="inlineStr">
+        <is>
+          <t>[[2212, 83], [257, 7033]]</t>
+        </is>
+      </c>
+      <c r="R97" t="n">
+        <v>0.9943652778898483</v>
+      </c>
+      <c r="S97" t="n">
+        <v>0.9981518959221709</v>
+      </c>
+      <c r="T97" t="n">
+        <v>0.9638344226579521</v>
+      </c>
+      <c r="U97" t="n">
+        <v>0.9647462277091907</v>
+      </c>
+      <c r="V97" t="n">
+        <v>2212</v>
+      </c>
+      <c r="W97" t="n">
+        <v>83</v>
+      </c>
+      <c r="X97" t="n">
+        <v>257</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>7033</v>
+      </c>
+      <c r="Z97" t="n">
+        <v>2.96991849862166</v>
+      </c>
+      <c r="AA97" t="n">
+        <v>0.6180048661800487</v>
+      </c>
+      <c r="AB97" t="n">
+        <v>0.4654563492063492</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>0.7503168567807351</v>
+      </c>
+      <c r="AD97" t="n">
+        <v>0.7517460317460317</v>
+      </c>
+      <c r="AE97" t="n">
+        <v>0.7510307643514114</v>
+      </c>
+      <c r="AF97" t="n">
+        <v>-0.06923830685181474</v>
+      </c>
+      <c r="AG97" t="n">
+        <v>-0.06923772879569712</v>
+      </c>
+      <c r="AH97" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI97" t="inlineStr">
+        <is>
+          <t>[[86, 394], [391, 1184]]</t>
+        </is>
+      </c>
+      <c r="AJ97" t="n">
+        <v>0.4216322751322751</v>
+      </c>
+      <c r="AK97" t="n">
+        <v>0.726719223586239</v>
+      </c>
+      <c r="AL97" t="n">
+        <v>0.1791666666666667</v>
+      </c>
+      <c r="AM97" t="n">
+        <v>0.7517460317460317</v>
+      </c>
+      <c r="AN97" t="n">
+        <v>86</v>
+      </c>
+      <c r="AO97" t="n">
+        <v>394</v>
+      </c>
+      <c r="AP97" t="n">
+        <v>391</v>
+      </c>
+      <c r="AQ97" t="n">
+        <v>1184</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>23</v>
+      </c>
+      <c r="D98" t="n">
+        <v>5e-05</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>0.747308423052565</v>
+      </c>
+      <c r="G98" t="b">
+        <v>0</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0.08434208759422966</v>
+      </c>
+      <c r="I98" t="n">
+        <v>0.9685967657798644</v>
+      </c>
+      <c r="J98" t="n">
+        <v>0.9680101670297749</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0.989357232880549</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0.9691358024691358</v>
+      </c>
+      <c r="M98" t="n">
+        <v>0.9791421245928903</v>
+      </c>
+      <c r="N98" t="n">
+        <v>0.9164531645758054</v>
+      </c>
+      <c r="O98" t="n">
+        <v>0.915653996282161</v>
+      </c>
+      <c r="P98" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q98" t="inlineStr">
+        <is>
+          <t>[[2219, 76], [225, 7065]]</t>
+        </is>
+      </c>
+      <c r="R98" t="n">
+        <v>0.9954929156542972</v>
+      </c>
+      <c r="S98" t="n">
+        <v>0.9985312014784259</v>
+      </c>
+      <c r="T98" t="n">
+        <v>0.966884531590414</v>
+      </c>
+      <c r="U98" t="n">
+        <v>0.9691358024691358</v>
+      </c>
+      <c r="V98" t="n">
+        <v>2219</v>
+      </c>
+      <c r="W98" t="n">
+        <v>76</v>
+      </c>
+      <c r="X98" t="n">
+        <v>225</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>7065</v>
+      </c>
+      <c r="Z98" t="n">
+        <v>2.854844876913549</v>
+      </c>
+      <c r="AA98" t="n">
+        <v>0.6116788321167883</v>
+      </c>
+      <c r="AB98" t="n">
+        <v>0.4548115079365079</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>0.7454200884396716</v>
+      </c>
+      <c r="AD98" t="n">
+        <v>0.7492063492063492</v>
+      </c>
+      <c r="AE98" t="n">
+        <v>0.747308423052565</v>
+      </c>
+      <c r="AF98" t="n">
+        <v>-0.09090908484368387</v>
+      </c>
+      <c r="AG98" t="n">
+        <v>-0.09090364812006069</v>
+      </c>
+      <c r="AH98" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI98" t="inlineStr">
+        <is>
+          <t>[[77, 403], [395, 1180]]</t>
+        </is>
+      </c>
+      <c r="AJ98" t="n">
+        <v>0.4326746031746032</v>
+      </c>
+      <c r="AK98" t="n">
+        <v>0.7400841460309429</v>
+      </c>
+      <c r="AL98" t="n">
+        <v>0.1604166666666667</v>
+      </c>
+      <c r="AM98" t="n">
+        <v>0.7492063492063492</v>
+      </c>
+      <c r="AN98" t="n">
+        <v>77</v>
+      </c>
+      <c r="AO98" t="n">
+        <v>403</v>
+      </c>
+      <c r="AP98" t="n">
+        <v>395</v>
+      </c>
+      <c r="AQ98" t="n">
+        <v>1180</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>24</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1.5e-05</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>0.7593114241001565</v>
+      </c>
+      <c r="G99" t="b">
+        <v>0</v>
+      </c>
+      <c r="H99" t="n">
+        <v>0.08463989851698007</v>
+      </c>
+      <c r="I99" t="n">
+        <v>0.9678664580073031</v>
+      </c>
+      <c r="J99" t="n">
+        <v>0.9667836681997902</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0.9886618141097424</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0.9688614540466393</v>
+      </c>
+      <c r="M99" t="n">
+        <v>0.9786614936954413</v>
+      </c>
+      <c r="N99" t="n">
+        <v>0.914420901992033</v>
+      </c>
+      <c r="O99" t="n">
+        <v>0.9136546343312459</v>
+      </c>
+      <c r="P99" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>[[2214, 81], [227, 7063]]</t>
+        </is>
+      </c>
+      <c r="R99" t="n">
+        <v>0.9955571095989073</v>
+      </c>
+      <c r="S99" t="n">
+        <v>0.9985680606321919</v>
+      </c>
+      <c r="T99" t="n">
+        <v>0.9647058823529412</v>
+      </c>
+      <c r="U99" t="n">
+        <v>0.9688614540466393</v>
+      </c>
+      <c r="V99" t="n">
+        <v>2214</v>
+      </c>
+      <c r="W99" t="n">
+        <v>81</v>
+      </c>
+      <c r="X99" t="n">
+        <v>227</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>7063</v>
+      </c>
+      <c r="Z99" t="n">
+        <v>3.066881872209609</v>
+      </c>
+      <c r="AA99" t="n">
+        <v>0.6257907542579075</v>
+      </c>
+      <c r="AB99" t="n">
+        <v>0.4611210317460318</v>
+      </c>
+      <c r="AC99" t="n">
+        <v>0.7487654320987654</v>
+      </c>
+      <c r="AD99" t="n">
+        <v>0.7701587301587302</v>
+      </c>
+      <c r="AE99" t="n">
+        <v>0.7593114241001565</v>
+      </c>
+      <c r="AF99" t="n">
+        <v>-0.08053849114735206</v>
+      </c>
+      <c r="AG99" t="n">
+        <v>-0.08037737783930687</v>
+      </c>
+      <c r="AH99" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI99" t="inlineStr">
+        <is>
+          <t>[[73, 407], [362, 1213]]</t>
+        </is>
+      </c>
+      <c r="AJ99" t="n">
+        <v>0.4277414021164021</v>
+      </c>
+      <c r="AK99" t="n">
+        <v>0.7420072212462632</v>
+      </c>
+      <c r="AL99" t="n">
+        <v>0.1520833333333333</v>
+      </c>
+      <c r="AM99" t="n">
+        <v>0.7701587301587302</v>
+      </c>
+      <c r="AN99" t="n">
+        <v>73</v>
+      </c>
+      <c r="AO99" t="n">
+        <v>407</v>
+      </c>
+      <c r="AP99" t="n">
+        <v>362</v>
+      </c>
+      <c r="AQ99" t="n">
+        <v>1213</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>25</v>
+      </c>
+      <c r="D100" t="n">
+        <v>1.5e-05</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>0.7577367927477336</v>
+      </c>
+      <c r="G100" t="b">
+        <v>0</v>
+      </c>
+      <c r="H100" t="n">
+        <v>0.06414638089446519</v>
+      </c>
+      <c r="I100" t="n">
+        <v>0.9790297339593115</v>
+      </c>
+      <c r="J100" t="n">
+        <v>0.9778544339546518</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0.9922233023191224</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0.9801097393689986</v>
+      </c>
+      <c r="M100" t="n">
+        <v>0.9861293216479194</v>
+      </c>
+      <c r="N100" t="n">
+        <v>0.9434767316141309</v>
+      </c>
+      <c r="O100" t="n">
+        <v>0.9431780627744841</v>
+      </c>
+      <c r="P100" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q100" t="inlineStr">
+        <is>
+          <t>[[2239, 56], [145, 7145]]</t>
+        </is>
+      </c>
+      <c r="R100" t="n">
+        <v>0.9973989498253194</v>
+      </c>
+      <c r="S100" t="n">
+        <v>0.9991416028349047</v>
+      </c>
+      <c r="T100" t="n">
+        <v>0.9755991285403051</v>
+      </c>
+      <c r="U100" t="n">
+        <v>0.9801097393689986</v>
+      </c>
+      <c r="V100" t="n">
+        <v>2239</v>
+      </c>
+      <c r="W100" t="n">
+        <v>56</v>
+      </c>
+      <c r="X100" t="n">
+        <v>145</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>7145</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>3.201292110823657</v>
+      </c>
+      <c r="AA100" t="n">
+        <v>0.6228710462287105</v>
+      </c>
+      <c r="AB100" t="n">
+        <v>0.4555952380952381</v>
+      </c>
+      <c r="AC100" t="n">
+        <v>0.7463054187192119</v>
+      </c>
+      <c r="AD100" t="n">
+        <v>0.7695238095238095</v>
+      </c>
+      <c r="AE100" t="n">
+        <v>0.7577367927477336</v>
+      </c>
+      <c r="AF100" t="n">
+        <v>-0.09229725642455364</v>
+      </c>
+      <c r="AG100" t="n">
+        <v>-0.09207697766989287</v>
+      </c>
+      <c r="AH100" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI100" t="inlineStr">
+        <is>
+          <t>[[68, 412], [363, 1212]]</t>
+        </is>
+      </c>
+      <c r="AJ100" t="n">
+        <v>0.4110886243386244</v>
+      </c>
+      <c r="AK100" t="n">
+        <v>0.733580177570053</v>
+      </c>
+      <c r="AL100" t="n">
+        <v>0.1416666666666667</v>
+      </c>
+      <c r="AM100" t="n">
+        <v>0.7695238095238095</v>
+      </c>
+      <c r="AN100" t="n">
+        <v>68</v>
+      </c>
+      <c r="AO100" t="n">
+        <v>412</v>
+      </c>
+      <c r="AP100" t="n">
+        <v>363</v>
+      </c>
+      <c r="AQ100" t="n">
+        <v>1212</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>26</v>
+      </c>
+      <c r="D101" t="n">
+        <v>1.5e-05</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>0.7472458293988039</v>
+      </c>
+      <c r="G101" t="b">
+        <v>0</v>
+      </c>
+      <c r="H101" t="n">
+        <v>0.05454964137708513</v>
+      </c>
+      <c r="I101" t="n">
+        <v>0.980490349504434</v>
+      </c>
+      <c r="J101" t="n">
+        <v>0.9795610425240056</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0.9929215822345593</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0.9813443072702333</v>
+      </c>
+      <c r="M101" t="n">
+        <v>0.9870989996550534</v>
+      </c>
+      <c r="N101" t="n">
+        <v>0.9473785103925056</v>
+      </c>
+      <c r="O101" t="n">
+        <v>0.9471046393498137</v>
+      </c>
+      <c r="P101" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q101" t="inlineStr">
+        <is>
+          <t>[[2244, 51], [136, 7154]]</t>
+        </is>
+      </c>
+      <c r="R101" t="n">
+        <v>0.9982381930062072</v>
+      </c>
+      <c r="S101" t="n">
+        <v>0.9994539090890602</v>
+      </c>
+      <c r="T101" t="n">
+        <v>0.9777777777777777</v>
+      </c>
+      <c r="U101" t="n">
+        <v>0.9813443072702333</v>
+      </c>
+      <c r="V101" t="n">
+        <v>2244</v>
+      </c>
+      <c r="W101" t="n">
+        <v>51</v>
+      </c>
+      <c r="X101" t="n">
+        <v>136</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>7154</v>
+      </c>
+      <c r="Z101" t="n">
+        <v>3.355111125611911</v>
+      </c>
+      <c r="AA101" t="n">
+        <v>0.6092457420924574</v>
+      </c>
+      <c r="AB101" t="n">
+        <v>0.4445337301587302</v>
+      </c>
+      <c r="AC101" t="n">
+        <v>0.7409488139825219</v>
+      </c>
+      <c r="AD101" t="n">
+        <v>0.7536507936507937</v>
+      </c>
+      <c r="AE101" t="n">
+        <v>0.7472458293988039</v>
+      </c>
+      <c r="AF101" t="n">
+        <v>-0.113224261495993</v>
+      </c>
+      <c r="AG101" t="n">
+        <v>-0.1131449270962976</v>
+      </c>
+      <c r="AH101" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI101" t="inlineStr">
+        <is>
+          <t>[[65, 415], [388, 1187]]</t>
+        </is>
+      </c>
+      <c r="AJ101" t="n">
+        <v>0.3991593915343915</v>
+      </c>
+      <c r="AK101" t="n">
+        <v>0.722205152130407</v>
+      </c>
+      <c r="AL101" t="n">
+        <v>0.1354166666666667</v>
+      </c>
+      <c r="AM101" t="n">
+        <v>0.7536507936507937</v>
+      </c>
+      <c r="AN101" t="n">
+        <v>65</v>
+      </c>
+      <c r="AO101" t="n">
+        <v>415</v>
+      </c>
+      <c r="AP101" t="n">
+        <v>388</v>
+      </c>
+      <c r="AQ101" t="n">
+        <v>1187</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>27</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1.5e-05</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>0.7620829435609604</v>
+      </c>
+      <c r="G102" t="b">
+        <v>0</v>
+      </c>
+      <c r="H102" t="n">
+        <v>0.05669132149294913</v>
+      </c>
+      <c r="I102" t="n">
+        <v>0.9798643714136672</v>
+      </c>
+      <c r="J102" t="n">
+        <v>0.9798959089808763</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0.9936013353734873</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0.9798353909465021</v>
+      </c>
+      <c r="M102" t="n">
+        <v>0.986670350162304</v>
+      </c>
+      <c r="N102" t="n">
+        <v>0.9459202084946554</v>
+      </c>
+      <c r="O102" t="n">
+        <v>0.9455359165649829</v>
+      </c>
+      <c r="P102" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q102" t="inlineStr">
+        <is>
+          <t>[[2249, 46], [147, 7143]]</t>
+        </is>
+      </c>
+      <c r="R102" t="n">
+        <v>0.9980123785530064</v>
+      </c>
+      <c r="S102" t="n">
+        <v>0.9993693542416082</v>
+      </c>
+      <c r="T102" t="n">
+        <v>0.9799564270152505</v>
+      </c>
+      <c r="U102" t="n">
+        <v>0.9798353909465021</v>
+      </c>
+      <c r="V102" t="n">
+        <v>2249</v>
+      </c>
+      <c r="W102" t="n">
+        <v>46</v>
+      </c>
+      <c r="X102" t="n">
+        <v>147</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>7143</v>
+      </c>
+      <c r="Z102" t="n">
+        <v>3.301499125441206</v>
+      </c>
+      <c r="AA102" t="n">
+        <v>0.6287104622871046</v>
+      </c>
+      <c r="AB102" t="n">
+        <v>0.4608531746031746</v>
+      </c>
+      <c r="AC102" t="n">
+        <v>0.7487745098039216</v>
+      </c>
+      <c r="AD102" t="n">
+        <v>0.7758730158730158</v>
+      </c>
+      <c r="AE102" t="n">
+        <v>0.7620829435609604</v>
+      </c>
+      <c r="AF102" t="n">
+        <v>-0.08193268387799232</v>
+      </c>
+      <c r="AG102" t="n">
+        <v>-0.08166475232566572</v>
+      </c>
+      <c r="AH102" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI102" t="inlineStr">
+        <is>
+          <t>[[70, 410], [353, 1222]]</t>
+        </is>
+      </c>
+      <c r="AJ102" t="n">
+        <v>0.4156587301587302</v>
+      </c>
+      <c r="AK102" t="n">
+        <v>0.737877354983045</v>
+      </c>
+      <c r="AL102" t="n">
+        <v>0.1458333333333333</v>
+      </c>
+      <c r="AM102" t="n">
+        <v>0.7758730158730158</v>
+      </c>
+      <c r="AN102" t="n">
+        <v>70</v>
+      </c>
+      <c r="AO102" t="n">
+        <v>410</v>
+      </c>
+      <c r="AP102" t="n">
+        <v>353</v>
+      </c>
+      <c r="AQ102" t="n">
+        <v>1222</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>resnet50_v4</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>2026-06-20 13:04:39</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>28</v>
+      </c>
+      <c r="D103" t="n">
+        <v>4.5e-06</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>val_f1</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>0.748898678414097</v>
+      </c>
+      <c r="G103" t="b">
+        <v>0</v>
+      </c>
+      <c r="H103" t="n">
+        <v>0.05400844431818931</v>
+      </c>
+      <c r="I103" t="n">
+        <v>0.9820552947313511</v>
+      </c>
+      <c r="J103" t="n">
+        <v>0.9822319051077221</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0.9944429008057794</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.9818930041152263</v>
+      </c>
+      <c r="M103" t="n">
+        <v>0.9881281060187742</v>
+      </c>
+      <c r="N103" t="n">
+        <v>0.9517193834851193</v>
+      </c>
+      <c r="O103" t="n">
+        <v>0.9513977330616403</v>
+      </c>
+      <c r="P103" t="n">
+        <v>9585</v>
+      </c>
+      <c r="Q103" t="inlineStr">
+        <is>
+          <t>[[2255, 40], [132, 7158]]</t>
+        </is>
+      </c>
+      <c r="R103" t="n">
+        <v>0.9981966522319947</v>
+      </c>
+      <c r="S103" t="n">
+        <v>0.9994122754129047</v>
+      </c>
+      <c r="T103" t="n">
+        <v>0.9825708061002179</v>
+      </c>
+      <c r="U103" t="n">
+        <v>0.9818930041152263</v>
+      </c>
+      <c r="V103" t="n">
+        <v>2255</v>
+      </c>
+      <c r="W103" t="n">
+        <v>40</v>
+      </c>
+      <c r="X103" t="n">
+        <v>132</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>7158</v>
+      </c>
+      <c r="Z103" t="n">
+        <v>3.194279748911985</v>
+      </c>
+      <c r="AA103" t="n">
+        <v>0.6116788321167883</v>
+      </c>
+      <c r="AB103" t="n">
+        <v>0.4475694444444445</v>
+      </c>
+      <c r="AC103" t="n">
+        <v>0.74235807860262</v>
+      </c>
+      <c r="AD103" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="AE103" t="n">
+        <v>0.748898678414097</v>
+      </c>
+      <c r="AF103" t="n">
+        <v>-0.1071123072610541</v>
+      </c>
+      <c r="AG103" t="n">
+        <v>-0.1070314715055289</v>
+      </c>
+      <c r="AH103" t="n">
+        <v>2055</v>
+      </c>
+      <c r="AI103" t="inlineStr">
+        <is>
+          <t>[[67, 413], [385, 1190]]</t>
+        </is>
+      </c>
+      <c r="AJ103" t="n">
+        <v>0.4210588624338625</v>
+      </c>
+      <c r="AK103" t="n">
+        <v>0.7325849420739675</v>
+      </c>
+      <c r="AL103" t="n">
+        <v>0.1395833333333333</v>
+      </c>
+      <c r="AM103" t="n">
+        <v>0.7555555555555555</v>
+      </c>
+      <c r="AN103" t="n">
+        <v>67</v>
+      </c>
+      <c r="AO103" t="n">
+        <v>413</v>
+      </c>
+      <c r="AP103" t="n">
+        <v>385</v>
+      </c>
+      <c r="AQ103" t="n">
+        <v>1190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>